<commit_message>
feat(products): make the product link optional in bulk import
Lets admins import a spreadsheet of products before every Amazon URL
is finalized. Two existing safeguards make this safe: imported rows
already always land as inactive, and the public "View on Amazon"
button already renders a graceful "Link unavailable" state instead of
a broken link. The single-product create/edit form is untouched and
still requires a valid link before a product can be saved, so there's
no way to activate a product without one.

- product_link column is now nullable (V24 migration)
- ProductImportValidator only enforces the https:// format when a
  link is actually provided, not that one exists
- ProductImportRowWriter no longer NPEs on a blank link
- Updated the .xlsx template's "How to use" notes to match, and
  removed its stray copy from the public storefront's static assets
  (it was leftover from before the admin/storefront app split and
  was never referenced there)
</commit_message>
<xml_diff>
--- a/admin/public/templates/product-list-template.xlsx
+++ b/admin/public/templates/product-list-template.xlsx
@@ -561,6 +561,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -653,10 +654,11 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Required. A full https:// product link.</t>
-        </is>
-      </c>
-    </row>
+          <t>Optional. A full https:// product link if you have one yet -- you can add it later, but the product cannot be published until it has one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>

</xml_diff>